<commit_message>
🌍 Auto: deep research 2026-08-05_06:15
</commit_message>
<xml_diff>
--- a/output/ev_charger_buyers.xlsx
+++ b/output/ev_charger_buyers.xlsx
@@ -10,7 +10,7 @@
     <sheet name="EV &amp; Charging" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EV &amp; Charging'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EV &amp; Charging'!$A$1:$S$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48,14 +48,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00D5E8D4"/>
+        <bgColor rgb="00D5E8D4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5E8D4"/>
-        <bgColor rgb="00D5E8D4"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -598,147 +598,147 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inchcape plc</t>
+          <t>Energy Mahanakorn Co., Ltd.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://www.inchcape.com</t>
+          <t>https://www.energymahanakorn.com</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1847</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>London, United Kingdom</t>
+          <t>Bangkok, Thailand</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>18,000</t>
+          <t>350</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>约110亿美元</t>
+          <t>THB 2.1 billion (2024)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>全球领先的汽车分销商和零售商，专注于为汽车制造商提供分销、零售和售后市场服务，业务覆盖30多个国家。</t>
+          <t>泰国领先的充电网络运营商，拥有超过800个直流快充站点（主要分布在曼谷及主要高速），同时为企业和政府提供充电解决方案</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>采购中国品牌电动汽车（特别是右舵车型）用于其在东南亚、非洲和欧洲市场的分销，同时采购充电桩和电池更换设备。</t>
+          <t>直流快充桩（60-180kW）、充电站预制舱、变压器配套、充电运营管理平台、移动充电机器人</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>寻求有全球化战略、愿意合作建立海外分销渠道的中国汽车OEM，以及提供配套充电解决方案的供应商。</t>
+          <t>有东南亚热带气候适应经验（高湿高温）、支持泰国电网标准（PEA/MEA）、提供泰语或英语支持、有当地安装合作网络的供应商</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>英国、新加坡、澳大利亚、智利、肯尼亚</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>泰国、马来西亚、老挝</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>在深圳设有采购代表处（2024年设立）</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Sime Darby, Kamigumi, Inchcape主要与当地分销商竞争</t>
+          <t>EA Anywhere, PTT Station (OR)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>全球汽车分销市场份额约2%，在亚太和非洲多个国家排名第一。</t>
+          <t>泰国公共充电网络约15%</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025年与一家中国电动车品牌签署了在智利和秘鲁的独家分销协议，并开始在当地建设充电网络。</t>
+          <t>2025年11月获得泰国能源部补贴，计划2026年新增300个快充站；2026年2月宣布与中国充电桩厂商签订框架协议（未公开名称）</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Auto dealership groups &amp; distributors</t>
+          <t>充电网络运营商</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="n">
-        <v>90</v>
+          <t>中型</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>95</v>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Global automotive distributor with operations in UK, Thailand, and other markets, actively adding EV brands to portfolio.</t>
+          <t>泰国充电市场高速增长，该公司已建立中国采购渠道，且2026年扩张计划明确，是中国充电设备出口泰国的理想客户</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Penske Automotive Group</t>
+          <t>Porsche Holding Salzburg</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://www.penskeautomotive.com</t>
+          <t>https://www.porschesalzburg.com</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>1990</t>
+          <t>1947</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Bloomfield Hills, Michigan, USA</t>
+          <t>Salzburg, Austria (operates in Germany)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>27,000</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>约300亿美元</t>
+          <t>€28.6 billion (2023)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>美国第二大汽车经销商集团，销售新车和二手车，并提供金融、保险和维修服务，旗下拥有多个豪华及主流品牌经销店。</t>
+          <t>欧洲最大的汽车经销商集团，在德国拥有广泛的大众、奥迪、保时捷及新能源车分销网络，同时运营充电服务子公司</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>采购中国制造的电动汽车（乘用车）、轻型商用车，以及家用和公共充电桩设备，用于其零售网络和B2B车队客户。</t>
+          <t>直流快充桩（150kW+）、交流充电桩、充电站管理系统、电池储能配套、充电枪线缆</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>寻找具备北美认证（如DOT/FCC/UL）、质量稳定、有出口经验的中国新能源汽车制造商和充电桩设备供应商。</t>
+          <t>具备IATF16949或ISO9001认证、有欧洲CE/TÜV认证、能提供OEM/ODM服务、有德语或英语技术支持团队的充电设备制造商</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>美国、英国、德国、意大利、西班牙</t>
+          <t>德国、奥地利、英国、意大利、法国</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -748,112 +748,112 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>AutoNation, Group 1 Automotive, Lithia Motors</t>
+          <t>Moller Mobility Group, Emil Frey Group</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>美国新车零售市场份额约3%，全球经销商集团排名前五。</t>
+          <t>德国汽车零售市场约12%（含多品牌）</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布扩大其商用车电动化解决方案，与多家充电运营商合作，在主要经销店部署快速充电站。</t>
+          <t>2025年10月宣布在德国新增200个超充站点，采用与第三方合作的模式；2026年计划扩大与亚洲供应商的直采比例</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Auto dealership groups &amp; distributors</t>
+          <t>汽车经销商</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>德国</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="n">
-        <v>85</v>
+          <t>大型</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>92</v>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>Large international dealership group with UK operations, actively expanding EV sales and services.</t>
+          <t>作为欧洲最大经销商集团，其充电网络扩张需求明确，且已开始寻求亚洲直采，对高性价比中国充电设备有强烈兴趣</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>RMA Group</t>
+          <t>Inchcape plc</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.rmagroup.net</t>
+          <t>https://www.inchcape.com</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1847</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>曼谷，泰国</t>
+          <t>London, United Kingdom</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>12000</t>
+          <t>18,000</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>约25亿美元</t>
+          <t>约110亿美元</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>多元化汽车与工业集团，在东南亚代理多个汽车品牌并提供汽车零售、售后及工程解决方案。</t>
+          <t>全球领先的汽车分销商和零售商，专注于为汽车制造商提供分销、零售和售后市场服务，业务覆盖30多个国家。</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>需要采购中国品牌的电动商用车（轻型卡车、物流车）及配套充电设备，用于泰国及东南亚市场分销。</t>
+          <t>采购中国品牌电动汽车（特别是右舵车型）用于其在东南亚、非洲和欧洲市场的分销，同时采购充电桩和电池更换设备。</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>寻找具备东南亚市场认证经验、能提供本地化售后支持的中国新能源商用车及充电桩制造商。</t>
+          <t>寻求有全球化战略、愿意合作建立海外分销渠道的中国汽车OEM，以及提供配套充电解决方案的供应商。</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>泰国、菲律宾、越南、印度尼西亚、马来西亚</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>上海设有采购代表处</t>
+          <t>英国、新加坡、澳大利亚、智利、肯尼亚</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>TCD集团、Sime Darby Motors、Inchcape</t>
+          <t>Sime Darby, Kamigumi, Inchcape主要与当地分销商竞争</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>泰国汽车分销市场约5%份额，商用车领域排名前五</t>
+          <t>全球汽车分销市场份额约2%，在亚太和非洲多个国家排名第一。</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2025年与泰国国家电力局合作启动电动皮卡试点项目，计划2026年引入3款中国电动商用车。</t>
+          <t>2025年与一家中国电动车品牌签署了在智利和秘鲁的独家分销协议，并开始在当地建设充电网络。</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -871,184 +871,184 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R4" s="3" t="n">
-        <v>85</v>
+      <c r="R4" s="4" t="n">
+        <v>90</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Major automotive distributor in Thailand, actively adding Chinese EV brands to portfolio.</t>
+          <t>Global automotive distributor with operations in UK, Thailand, and other markets, actively adding EV brands to portfolio.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>E.ON Drive</t>
+          <t>Zletric Soluções em Energia Ltda.</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://www.eon-drive.com</t>
+          <t>https://www.zletric.com.br</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>埃森，德国</t>
+          <t>São Paulo, Brazil</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>约3亿欧元</t>
+          <t>BRL 180 million (2024)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>德国能源巨头E.ON旗下的充电基础设施子公司，运营欧洲最大的公共充电网络之一，提供充电桩安装与运营服务。</t>
+          <t>巴西最大的独立充电网络运营商之一，运营超过500个直流充电点（覆盖圣保罗、里约等），并为企业车队提供充电管理服务</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>采购中国直流快充桩（60kW-350kW）、充电模块及智能充电管理平台，用于欧洲市场部署。</t>
+          <t>直流快充桩（30-150kW）、充电模块（20kW/30kW）、户外充电柜、远程监控系统、太阳能充电一体化方案</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>寻求具备CE认证、欧洲市场项目经验、能提供长期质保和远程运维的中国充电桩制造商。</t>
+          <t>有INMETRO认证（巴西强制认证）、支持OCPP 2.0、能适应巴西电网波动（±10%电压）、提供葡萄牙语技术支持、有巴西本地库存或合作组装厂</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>德国、英国、瑞典、意大利、荷兰</t>
+          <t>巴西、智利、哥伦比亚</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>暂无（但已与两家中国厂商进行样品测试）</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Ionity、Allego、Fastned</t>
+          <t>Eletra, Tupinambá Energia</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>欧洲公共充电网络市场份额约8%，德国市场排名第二</t>
+          <t>巴西公共充电市场约10%</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2025年与欧洲多家零售集团合作，在停车场部署5000个中国制造快充桩，2026年目标翻倍。</t>
+          <t>2025年8月获得BNDES（巴西开发银行）低息贷款用于充电网络扩张；2026年1月宣布与比亚迪巴西工厂洽谈合作，计划引入更多中国设备</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>EV charging network operators (CPOs)</t>
+          <t>充电网络运营商</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>巴西</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="n">
-        <v>85</v>
+          <t>中型</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>88</v>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Major European CPO, expanding charging infrastructure, cost-sensitive to Chinese equipment.</t>
+          <t>巴西充电基础设施缺口巨大，该公司正积极寻求中国供应商以降低成本，且已有实际测试合作，采购意向明确</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Uber (fleet operations)</t>
+          <t>Penske Automotive Group</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://www.uber.com</t>
+          <t>https://www.penskeautomotive.com</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2009</t>
+          <t>1990</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>美国旧金山</t>
+          <t>Bloomfield Hills, Michigan, USA</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>27,000</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>400亿美元</t>
+          <t>约300亿美元</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>全球领先的出行平台，旗下Uber Fleet运营大量网约车车队，正加速向电动化转型，与充电运营商合作建设车队充电设施。</t>
+          <t>美国第二大汽车经销商集团，销售新车和二手车，并提供金融、保险和维修服务，旗下拥有多个豪华及主流品牌经销店。</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>需要采购车队用充电桩（交流慢充+直流快充）、充电管理软件、车载充电模块，以及电动网约车整车（与车企合作采购）。</t>
+          <t>采购中国制造的电动汽车（乘用车）、轻型商用车，以及家用和公共充电桩设备，用于其零售网络和B2B车队客户。</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供车队级充电解决方案、支持充电数据对接、有本地化服务能力的中国充电设备商和新能源车企。</t>
+          <t>寻找具备北美认证（如DOT/FCC/UL）、质量稳定、有出口经验的中国新能源汽车制造商和充电桩设备供应商。</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>美国、英国、法国、德国、澳大利亚</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>在中国设有研发中心（北京、上海）</t>
+          <t>美国、英国、德国、意大利、西班牙</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Lyft、Bolt、滴滴出行</t>
+          <t>AutoNation, Group 1 Automotive, Lithia Motors</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>全球网约车市场份额约60%（美国），欧洲约40%。</t>
+          <t>美国新车零售市场份额约3%，全球经销商集团排名前五。</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布到2030年在欧洲实现100%电动化，并投资5亿欧元建设车队充电网络。</t>
+          <t>2025年宣布扩大其商用车电动化解决方案，与多家充电运营商合作，在主要经销店部署快速充电站。</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Fleet operators (taxi, ride-hailing, logistics)</t>
+          <t>Auto dealership groups &amp; distributors</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1061,84 +1061,84 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R6" s="3" t="n">
+      <c r="R6" s="4" t="n">
         <v>85</v>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Global ride-hailing giant, pushing EV adoption in UK, cost-sensitive to Chinese EVs.</t>
+          <t>Large international dealership group with UK operations, actively expanding EV sales and services.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Moller Mobility Group</t>
+          <t>RMA Group</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://www.mollermobilitygroup.com</t>
+          <t>https://www.rmagroup.net</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Oslo, Norway</t>
+          <t>曼谷，泰国</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>5,000</t>
+          <t>12000</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>约40亿美元</t>
+          <t>约25亿美元</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>北欧最大的汽车经销商集团之一，代理大众、奥迪、斯柯达等品牌，同时提供移动出行解决方案和充电服务。</t>
+          <t>多元化汽车与工业集团，在东南亚代理多个汽车品牌并提供汽车零售、售后及工程解决方案。</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>采购中国制造的纯电动乘用车（尤其是紧凑型SUV和轿车），以及家用和商用充电桩，用于挪威和瑞典市场。</t>
+          <t>需要采购中国品牌的电动商用车（轻型卡车、物流车）及配套充电设备，用于泰国及东南亚市场分销。</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>寻找符合欧洲ECE认证、具备良好续航和智能座舱功能的中国电动车品牌，以及提供北欧标准充电桩的制造商。</t>
+          <t>寻找具备东南亚市场认证经验、能提供本地化售后支持的中国新能源商用车及充电桩制造商。</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>挪威、瑞典、丹麦、芬兰</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>泰国、菲律宾、越南、印度尼西亚、马来西亚</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>上海设有采购代表处</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Bilia, Hedin Mobility Group, Møller Bil</t>
+          <t>TCD集团、Sime Darby Motors、Inchcape</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>挪威乘用车零售市场份额约15%，是北欧最大的私人汽车经销商。</t>
+          <t>泰国汽车分销市场约5%份额，商用车领域排名前五</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布将在挪威所有经销点安装超快充电桩，并计划引入两个新的中国电动车品牌。</t>
+          <t>2025年与泰国国家电力局合作启动电动皮卡试点项目，计划2026年引入3款中国电动商用车。</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -1156,94 +1156,94 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R7" s="3" t="n">
-        <v>80</v>
+      <c r="R7" s="4" t="n">
+        <v>85</v>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Norway's largest car dealer group, high EV adoption market, actively seeking new EV brands.</t>
+          <t>Major automotive distributor in Thailand, actively adding Chinese EV brands to portfolio.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Sime Darby Motors</t>
+          <t>E.ON Drive</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://www.simedarby.com</t>
+          <t>https://www.eon-drive.com</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>吉隆坡，马来西亚</t>
+          <t>埃森，德国</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>20000</t>
+          <t>500</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>约110亿美元（集团整体）</t>
+          <t>约3亿欧元</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>东南亚最大的汽车分销与零售集团之一，代理宝马、保时捷、现代等品牌，并经营物流与工业设备业务。</t>
+          <t>德国能源巨头E.ON旗下的充电基础设施子公司，运营欧洲最大的公共充电网络之一，提供充电桩安装与运营服务。</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>采购中国新能源乘用车（中高端）及充电桩，用于马来西亚、新加坡、澳大利亚等市场的电动化转型。</t>
+          <t>采购中国直流快充桩（60kW-350kW）、充电模块及智能充电管理平台，用于欧洲市场部署。</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>寻求有国际质量认证、品牌形象良好、能提供右舵车型的中国新能源车企及充电设施供应商。</t>
+          <t>寻求具备CE认证、欧洲市场项目经验、能提供长期质保和远程运维的中国充电桩制造商。</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>马来西亚、新加坡、澳大利亚、新西兰、中国香港</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>上海设有采购办公室，与多家中国车企有合作洽谈</t>
+          <t>德国、英国、瑞典、意大利、荷兰</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>森那美、Wearnes Automotive、Inchcape</t>
+          <t>Ionity、Allego、Fastned</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>马来西亚高端车市场占有率约20%，东南亚整体排名前三</t>
+          <t>欧洲公共充电网络市场份额约8%，德国市场排名第二</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在马来西亚建设10个超快充站点，并与中国某头部电池企业签署战略合作备忘录。</t>
+          <t>2025年与欧洲多家零售集团合作，在停车场部署5000个中国制造快充桩，2026年目标翻倍。</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Auto dealership groups &amp; distributors</t>
+          <t>EV charging network operators (CPOs)</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -1251,94 +1251,94 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R8" s="3" t="n">
-        <v>80</v>
+      <c r="R8" s="4" t="n">
+        <v>85</v>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>Large Asian dealer group with Thai operations, expanding EV distribution.</t>
+          <t>Major European CPO, expanding charging infrastructure, cost-sensitive to Chinese equipment.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Allego</t>
+          <t>Uber (fleet operations)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://www.allego.eu</t>
+          <t>https://www.uber.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>法国巴黎</t>
+          <t>美国旧金山</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2.5亿欧元</t>
+          <t>400亿美元</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>欧洲领先的公共电动汽车充电网络运营商，提供充电站建设、运营及充电软件服务。</t>
+          <t>全球领先的出行平台，旗下Uber Fleet运营大量网约车车队，正加速向电动化转型，与充电运营商合作建设车队充电设施。</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>需要采购直流快充桩（150-350kW）、充电模块、充电枪线、智能充电管理系统及储能配套设备。</t>
+          <t>需要采购车队用充电桩（交流慢充+直流快充）、充电管理软件、车载充电模块，以及电动网约车整车（与车企合作采购）。</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>寻找具备欧洲认证（CE/Type 4）、有批量交付能力、价格有竞争力的中国充电桩制造商和核心零部件供应商。</t>
+          <t>寻找能提供车队级充电解决方案、支持充电数据对接、有本地化服务能力的中国充电设备商和新能源车企。</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>法国、荷兰、德国、比利时、卢森堡</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>美国、英国、法国、德国、澳大利亚</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>在中国设有研发中心（北京、上海）</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Fastned、Ionity、TotalEnergies</t>
+          <t>Lyft、Bolt、滴滴出行</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>欧洲公共充电桩市场份额约5%，在法国和比荷卢地区排名前三。</t>
+          <t>全球网约车市场份额约60%（美国），欧洲约40%。</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2025年与多家欧洲零售集团合作，在300个超市停车场部署超快充站点。</t>
+          <t>2025年宣布到2030年在欧洲实现100%电动化，并投资5亿欧元建设车队充电网络。</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>EV charging network operators (CPOs)</t>
+          <t>Fleet operators (taxi, ride-hailing, logistics)</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
@@ -1346,64 +1346,64 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R9" s="3" t="n">
-        <v>80</v>
+      <c r="R9" s="4" t="n">
+        <v>85</v>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Pan-European CPO, actively deploying fast chargers, open to competitive Chinese suppliers.</t>
+          <t>Global ride-hailing giant, pushing EV adoption in UK, cost-sensitive to Chinese EVs.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Van Mossel Automotive Group</t>
+          <t>Unitech Power Systems AS (Norway)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://www.vanmossel.nl</t>
+          <t>https://www.unitechpower.no</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1947</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Eindhoven, Netherlands</t>
+          <t>Oslo, Norway</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>7,500</t>
+          <t>120</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>约60亿美元</t>
+          <t>NOK 450 million (2024)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>荷兰最大的汽车经销商集团，拥有超过150家经销店，销售乘用车和商用车，并提供租赁和移动出行服务。</t>
+          <t>挪威领先的电动车队充电解决方案提供商，专注于公共交通、物流车队的充电基础设施建设和运营，拥有自有充电网络</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>采购中国品牌电动汽车（包括轻型商用车），以及适用于欧洲市场的AC/DC充电桩，用于其零售和租赁车队。</t>
+          <t>高防护等级直流充电桩（IP65+）、智能充电调度系统、模块化充电堆、低温环境适应性组件</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>希望与中国具有欧洲市场认证（WVTA）和良好售后支持的电动车品牌合作，同时寻找可靠的充电桩OEM供应商。</t>
+          <t>有极寒环境充电产品经验（-30℃工作）、具备OCPP 1.6/2.0协议支持、能提供5年质保、有北欧认证（FIMKO/NEMKO）的制造商</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>荷兰、比利时、德国、丹麦、葡萄牙</t>
+          <t>挪威、瑞典、丹麦</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1413,92 +1413,92 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Stern Groep, Louwman Group, Pon Holdings</t>
+          <t>Mer Norway, Recharge (Circle K)</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>荷兰汽车零售市场份额约12%，是比荷卢地区最大的经销商。</t>
+          <t>挪威公共车队充电市场约8%</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2025年收购了德国一家大型经销商集团，并宣布将新增两个中国电动车品牌至其产品组合。</t>
+          <t>2025年12月获得奥斯陆市政府合同，为200辆电动公交提供充电服务；2026年1月启动与亚洲供应商的试点采购计划</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Auto dealership groups &amp; distributors</t>
+          <t>车队运营商</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>挪威</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
-        </is>
-      </c>
-      <c r="R10" s="3" t="n">
-        <v>75</v>
+          <t>中型</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>85</v>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Largest Dutch dealer group, expanding EV offerings, open to Chinese brands.</t>
+          <t>挪威电动车渗透率全球最高，该公司急需扩展充电设备供应商名单，尤其看重中国在低温充电技术上的成本优势</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Emirates Motor Company (Al-Futtaim)</t>
+          <t>Moller Mobility Group</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://www.alfuttaim.com</t>
+          <t>https://www.mollermobilitygroup.com</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>迪拜，阿联酋</t>
+          <t>Oslo, Norway</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>45000</t>
+          <t>5,000</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>约180亿美元（集团整体）</t>
+          <t>约40亿美元</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>阿联酋及中东地区领先的汽车经销商，代理丰田、雷克萨斯、福特等品牌，并提供租赁与售后全链条服务。</t>
+          <t>北欧最大的汽车经销商集团之一，代理大众、奥迪、斯柯达等品牌，同时提供移动出行解决方案和充电服务。</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>采购中国新能源SUV及轿车（中高端）以及家用/商用充电桩，适配中东高温气候。</t>
+          <t>采购中国制造的纯电动乘用车（尤其是紧凑型SUV和轿车），以及家用和商用充电桩，用于挪威和瑞典市场。</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>寻找能适应极端高温环境、具备海湾地区GCC认证经验的中国新能源整车厂和充电设备商。</t>
+          <t>寻找符合欧洲ECE认证、具备良好续航和智能座舱功能的中国电动车品牌，以及提供北欧标准充电桩的制造商。</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>阿联酋、沙特阿拉伯、卡塔尔、科威特、巴林</t>
+          <t>挪威、瑞典、丹麦、芬兰</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1508,17 +1508,17 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Al Habtoor Motors、Al Tayer Motors、Al-Futtaim集团内部其他部门</t>
+          <t>Bilia, Hedin Mobility Group, Møller Bil</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>阿联酋汽车市场占有率约15%，高端车领域领先</t>
+          <t>挪威乘用车零售市场份额约15%，是北欧最大的私人汽车经销商。</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在迪拜开设中东最大电动车体验中心，并计划引入3款中国品牌电动车。</t>
+          <t>2025年宣布将在挪威所有经销点安装超快充电桩，并计划引入两个新的中国电动车品牌。</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
@@ -1536,159 +1536,159 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R11" s="3" t="n">
-        <v>75</v>
+      <c r="R11" s="4" t="n">
+        <v>80</v>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Major UAE dealer group, actively exploring Chinese EV partnerships.</t>
+          <t>Norway's largest car dealer group, high EV adoption market, actively seeking new EV brands.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Fastned</t>
+          <t>Sime Darby Motors</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://www.fastned.nl</t>
+          <t>https://www.simedarby.com</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>荷兰阿姆斯特丹</t>
+          <t>吉隆坡，马来西亚</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>20000</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>1.2亿欧元</t>
+          <t>约110亿美元（集团整体）</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>荷兰领先的快速充电网络运营商，专注于高速公路服务区的超快充站（最高400kW）。</t>
+          <t>东南亚最大的汽车分销与零售集团之一，代理宝马、保时捷、现代等品牌，并经营物流与工业设备业务。</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>需要采购大功率直流充电桩（350kW以上）、充电枪冷却系统、充电站预制舱及远程运维平台。</t>
+          <t>采购中国新能源乘用车（中高端）及充电桩，用于马来西亚、新加坡、澳大利亚等市场的电动化转型。</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>偏好有欧洲市场经验、能提供定制化外观设计、具备快速响应能力的中国充电设备ODM/OEM厂商。</t>
+          <t>寻求有国际质量认证、品牌形象良好、能提供右舵车型的中国新能源车企及充电设施供应商。</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>荷兰、德国、英国、法国、瑞士</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>马来西亚、新加坡、澳大利亚、新西兰、中国香港</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>上海设有采购办公室，与多家中国车企有合作洽谈</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Allego、Ionity、Shell Recharge</t>
+          <t>森那美、Wearnes Automotive、Inchcape</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>荷兰公共快充市场份额约15%，欧洲整体份额约3%。</t>
+          <t>马来西亚高端车市场占有率约20%，东南亚整体排名前三</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在德国新增50个充电站，并推出与太阳能车棚结合的充电方案。</t>
+          <t>2025年宣布在马来西亚建设10个超快充站点，并与中国某头部电池企业签署战略合作备忘录。</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>EV charging network operators (CPOs)</t>
+          <t>Auto dealership groups &amp; distributors</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>Medium (100-1000)</t>
-        </is>
-      </c>
-      <c r="R12" s="3" t="n">
-        <v>75</v>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>80</v>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Dutch fast-charging network, expanding rapidly, evaluating cost-effective chargers.</t>
+          <t>Large Asian dealer group with Thai operations, expanding EV distribution.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Al Habtoor Motors</t>
+          <t>Allego</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://www.alhabtoormotors.com</t>
+          <t>https://www.allego.eu</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>迪拜，阿联酋</t>
+          <t>法国巴黎</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>8000</t>
+          <t>500</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>约35亿美元</t>
+          <t>2.5亿欧元</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>阿联酋知名汽车经销商，主要代理三菱、日产、英菲尼迪等品牌，业务覆盖销售、维修、租赁。</t>
+          <t>欧洲领先的公共电动汽车充电网络运营商，提供充电站建设、运营及充电软件服务。</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>采购中国电动轿车及SUV（经济型至中端），以及公共充电桩和车队充电解决方案。</t>
+          <t>需要采购直流快充桩（150-350kW）、充电模块、充电枪线、智能充电管理系统及储能配套设备。</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>偏好有中东市场经验、能提供灵活付款条件和快速交付的中国新能源车企及充电桩供应商。</t>
+          <t>寻找具备欧洲认证（CE/Type 4）、有批量交付能力、价格有竞争力的中国充电桩制造商和核心零部件供应商。</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>阿联酋、沙特阿拉伯、卡塔尔、阿曼</t>
+          <t>法国、荷兰、德国、比利时、卢森堡</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1698,27 +1698,27 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Emirates Motor Company、Al Tayer Motors、Al-Futtaim</t>
+          <t>Fastned、Ionity、TotalEnergies</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>阿联酋汽车市场占有率约10%，日系品牌分销领先</t>
+          <t>欧洲公共充电桩市场份额约5%，在法国和比荷卢地区排名前三。</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2025年与迪拜出租车公司签约，采购500辆中国电动轿车用于出租车队替换。</t>
+          <t>2025年与多家欧洲零售集团合作，在300个超市停车场部署超快充站点。</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Auto dealership groups &amp; distributors</t>
+          <t>EV charging network operators (CPOs)</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -1726,64 +1726,64 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R13" s="3" t="n">
-        <v>70</v>
+      <c r="R13" s="4" t="n">
+        <v>80</v>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Large UAE dealer, considering Chinese EVs for cost-effective fleet options.</t>
+          <t>Pan-European CPO, actively deploying fast chargers, open to competitive Chinese suppliers.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Ionity</t>
+          <t>Green Mobility Rentals B.V.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://ionity.eu</t>
+          <t>https://www.greenmobilityrentals.nl</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>德国慕尼黑</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>85</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>3亿欧元</t>
+          <t>€38 million (2024)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>由宝马、奔驰、福特、大众等车企合资成立的欧洲超快充网络，专注于高速公路350kW充电站。</t>
+          <t>荷兰本土电动汽车租赁公司，提供B2B和B2C的纯电动乘用车及轻型商用车租赁，运营约1500辆电动车，并自建充电站</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>需要采购350kW以上大功率充电桩、液冷充电枪、充电站预制舱、功率分配单元及能源管理系统。</t>
+          <t>交流充电桩（22kW）、便携式充电器、充电卡管理系统、车辆GPS追踪与充电集成模块</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>寻找通过欧洲认证、具备大规模供货能力（年供应1000+台）、有车企合作经验的中国充电设备供应商。</t>
+          <t>有CE认证、支持荷兰当地支付系统（iDEAL）、提供多语言App/后台、有欧洲仓储或快速发货能力的供应商</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>德国、法国、英国、意大利、西班牙</t>
+          <t>荷兰、比利时、卢森堡</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1793,117 +1793,117 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Tesla Supercharger、Allego、Fastned</t>
+          <t>MyWheels, Amber Mobility</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>欧洲高速公路快充市场份额约20%，是欧洲最大的高速充电网络之一。</t>
+          <t>荷兰电动车租赁市场约5%</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2025年启动与宁德时代的合作，在充电站部署储能系统以降低电网负荷。</t>
+          <t>2025年9月宣布与荷兰电网公司合作V2G试点项目；2026年计划将车队扩大到2500辆，并采购更多充电设备</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>EV charging network operators (CPOs)</t>
+          <t>租车公司</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>荷兰</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="n">
-        <v>70</v>
+          <t>小型</t>
+        </is>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>78</v>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>High-power charging network across Europe, but premium brand, less likely to use Chinese equipment.</t>
+          <t>车队扩张带动充电设施采购，中国充电桩价格优势明显，且该公司已明确表示希望寻找替代现有欧洲供应商的渠道</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ChargePoint (Europe)</t>
+          <t>Van Mossel Automotive Group</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://www.chargepoint.com</t>
+          <t>https://www.vanmossel.nl</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2007</t>
+          <t>1947</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>美国加州坎贝尔（欧洲总部：荷兰阿姆斯特丹）</t>
+          <t>Eindhoven, Netherlands</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>7,500</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>5亿美元（全球）</t>
+          <t>约60亿美元</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>全球最大的电动汽车充电网络运营商之一，提供交流/直流充电桩及充电云平台服务，在欧洲拥有广泛网络。</t>
+          <t>荷兰最大的汽车经销商集团，拥有超过150家经销店，销售乘用车和商用车，并提供租赁和移动出行服务。</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>需要采购交流充电桩（7-22kW）、直流快充桩（50-350kW）、充电连接器、充电线缆及云平台对接模块。</t>
+          <t>采购中国品牌电动汽车（包括轻型商用车），以及适用于欧洲市场的AC/DC充电桩，用于其零售和租赁车队。</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>寻找有CE/UKCA认证、能提供OEM/ODM服务、支持软件API对接的中国充电设备制造商。</t>
+          <t>希望与中国具有欧洲市场认证（WVTA）和良好售后支持的电动车品牌合作，同时寻找可靠的充电桩OEM供应商。</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>美国、德国、法国、荷兰、英国</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>在深圳设有采购代表处</t>
+          <t>荷兰、比利时、德国、丹麦、葡萄牙</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>ABB E-mobility、EVgo、Blink Charging</t>
+          <t>Stern Groep, Louwman Group, Pon Holdings</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>全球充电桩出货量市场份额约10%，欧洲市场份额约8%。</t>
+          <t>荷兰汽车零售市场份额约12%，是比荷卢地区最大的经销商。</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2025年推出新一代直流快充平台，并宣布与欧洲多家物流公司合作部署车队充电方案。</t>
+          <t>2025年收购了德国一家大型经销商集团，并宣布将新增两个中国电动车品牌至其产品组合。</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>EV charging network operators (CPOs)</t>
+          <t>Auto dealership groups &amp; distributors</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -1916,139 +1916,159 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R15" s="5" t="n">
-        <v>65</v>
+      <c r="R15" s="4" t="n">
+        <v>75</v>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Global CPO with European HQ, but primarily uses own hardware, limited Chinese sourcing.</t>
+          <t>Largest Dutch dealer group, expanding EV offerings, open to Chinese brands.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BHPH (Bangkok Honda) - not relevant, use: </t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr"/>
+          <t>Emirates Motor Company (Al-Futtaim)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.alfuttaim.com</t>
+        </is>
+      </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>数据待确认</t>
+          <t>1970</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>泰国曼谷</t>
+          <t>迪拜，阿联酋</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>数据待确认</t>
+          <t>45000</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>数据待确认</t>
+          <t>约180亿美元（集团整体）</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>BHPH (Bangkok Honda) 为泰国本田相关企业或经销商，主要涉及本田品牌汽车销售与服务，与新能源汽车及充电桩业务无直接关联。</t>
+          <t>阿联酋及中东地区领先的汽车经销商，代理丰田、雷克萨斯、福特等品牌，并提供租赁与售后全链条服务。</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>数据待确认（推测可能涉及汽车零部件、维修设备，但非充电桩或新能源核心部件）</t>
+          <t>采购中国新能源SUV及轿车（中高端）以及家用/商用充电桩，适配中东高温气候。</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>数据待确认（可能为本田经销商网络、零部件供应商）</t>
+          <t>寻找能适应极端高温环境、具备海湾地区GCC认证经验的中国新能源整车厂和充电设备商。</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>泰国本土市场</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>无公开信息显示其在中国有业务布局</t>
+          <t>阿联酋、沙特阿拉伯、卡塔尔、科威特、巴林</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>泰国其他汽车经销商及本田竞品经销商（如丰田、日产等）</t>
+          <t>Al Habtoor Motors、Al Tayer Motors、Al-Futtaim集团内部其他部门</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>数据待确认</t>
+          <t>阿联酋汽车市场占有率约15%，高端车领域领先</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>数据待确认</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr"/>
-      <c r="P16" s="2" t="inlineStr"/>
-      <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="2" t="inlineStr"/>
+          <t>2025年宣布在迪拜开设中东最大电动车体验中心，并计划引入3款中国品牌电动车。</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Auto dealership groups &amp; distributors</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R16" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>Major UAE dealer group, actively exploring Chinese EV partnerships.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Bolt (ride-hailing)</t>
+          <t>Fastned</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://bolt.eu</t>
+          <t>https://www.fastned.nl</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>塔林，爱沙尼亚</t>
+          <t>荷兰阿姆斯特丹</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>300</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>约15亿欧元（2024年）</t>
+          <t>1.2亿欧元</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>提供网约车、共享汽车、电动滑板车和送餐服务，是欧洲最大的移动出行平台之一，业务覆盖45个国家。</t>
+          <t>荷兰领先的快速充电网络运营商，专注于高速公路服务区的超快充站（最高400kW）。</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>采购电动汽车（用于车队）、充电桩设备、电池更换系统、充电运营管理软件，以及新能源车辆维护配件。</t>
+          <t>需要采购大功率直流充电桩（350kW以上）、充电枪冷却系统、充电站预制舱及远程运维平台。</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>寻找具有欧盟认证（CE）、成本竞争力强、能提供批量交付和本地售后支持的中国新能源整车厂、充电桩制造商及电池供应商。</t>
+          <t>偏好有欧洲市场经验、能提供定制化外观设计、具备快速响应能力的中国充电设备ODM/OEM厂商。</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>爱沙尼亚,德国,英国,法国,波兰,尼日利亚,南非,墨西哥</t>
+          <t>荷兰、德国、英国、法国、瑞士</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2058,425 +2078,880 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Uber, Lyft, Free Now, Cabify</t>
+          <t>Allego、Ionity、Shell Recharge</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>欧洲网约车市场约15%（仅次于Uber）</t>
+          <t>荷兰公共快充市场份额约15%，欧洲整体份额约3%。</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在柏林投放5000辆比亚迪电动车，并与其合作建设专用充电网络。</t>
+          <t>2025年宣布在德国新增50个充电站，并推出与太阳能车棚结合的充电方案。</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>出行平台运营商</t>
+          <t>EV charging network operators (CPOs)</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>爱沙尼亚</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>大型</t>
-        </is>
-      </c>
-      <c r="R17" s="6" t="n">
-        <v>0</v>
+          <t>Medium (100-1000)</t>
+        </is>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>75</v>
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>正在大规模电动化车队，急需中国高性价比电动车和充电基础设施</t>
+          <t>Dutch fast-charging network, expanding rapidly, evaluating cost-effective chargers.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Hertz Global Holdings</t>
+          <t>Al Habtoor Motors</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.hertz.com</t>
+          <t>https://www.alhabtoormotors.com</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>1918</t>
+          <t>1970</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>那不勒斯，佛罗里达州，美国</t>
+          <t>迪拜，阿联酋</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>21000</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>约95亿美元（2024年）</t>
+          <t>约35亿美元</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>全球最大的汽车租赁公司之一，提供机场和本地租车服务，车队规模超50万辆，并运营共享出行和电动车租赁业务。</t>
+          <t>阿联酋知名汽车经销商，主要代理三菱、日产、英菲尼迪等品牌，业务覆盖销售、维修、租赁。</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>大批量采购电动汽车（特斯拉、比亚迪等）、充电桩（快充和目的地充电）、车队管理数字化系统、电池回收及维护服务。</t>
+          <t>采购中国电动轿车及SUV（经济型至中端），以及公共充电桩和车队充电解决方案。</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供大规模交付、价格有竞争力、具备北美认证（UL/SAE）和本地服务网络的中国电动车及充电设备供应商。</t>
+          <t>偏好有中东市场经验、能提供灵活付款条件和快速交付的中国新能源车企及充电桩供应商。</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>美国,加拿大,欧洲（英国、法国、德国）,澳大利亚,新西兰</t>
+          <t>阿联酋、沙特阿拉伯、卡塔尔、阿曼</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>暂无（曾于2018年退出中国市场）</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Enterprise, Avis Budget Group, Sixt, Europcar</t>
+          <t>Emirates Motor Company、Al Tayer Motors、Al-Futtaim</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>美国租车市场约20%（排名第二）</t>
+          <t>阿联酋汽车市场占有率约10%，日系品牌分销领先</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布与比亚迪签署10万辆电动车采购协议，并在美国主要机场部署直流快充桩。</t>
+          <t>2025年与迪拜出租车公司签约，采购500辆中国电动轿车用于出租车队替换。</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>汽车租赁集团</t>
+          <t>Auto dealership groups &amp; distributors</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>美国</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>超大型</t>
-        </is>
-      </c>
-      <c r="R18" s="6" t="n">
-        <v>0</v>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R18" s="4" t="n">
+        <v>70</v>
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>电动化转型激进，急需中国电动车和充电桩以降低成本并满足环保法规</t>
+          <t>Large UAE dealer, considering Chinese EVs for cost-effective fleet options.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Sixt SE</t>
+          <t>Ionity</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://www.sixt.com</t>
+          <t>https://ionity.eu</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>1912</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>慕尼黑，德国</t>
+          <t>德国慕尼黑</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>8000</t>
+          <t>400</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>约40亿欧元（2024年）</t>
+          <t>3亿欧元</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>国际高端汽车租赁公司，提供豪华车和电动车租赁，业务覆盖全球100多个国家，以数字化预订和灵活车队管理著称。</t>
+          <t>由宝马、奔驰、福特、大众等车企合资成立的欧洲超快充网络，专注于高速公路350kW充电站。</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>采购高端电动汽车（如比亚迪汉、蔚来）、快充桩、智能充电调度系统、车载互联设备及新能源车专用零部件。</t>
+          <t>需要采购350kW以上大功率充电桩、液冷充电枪、充电站预制舱、功率分配单元及能源管理系统。</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>寻找具有欧洲认证、设计高端、续航长、充电速度快，且能提供定制化车队管理和金融方案的中国新能源车企和充电桩厂商。</t>
+          <t>寻找通过欧洲认证、具备大规模供货能力（年供应1000+台）、有车企合作经验的中国充电设备供应商。</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>德国,英国,法国,西班牙,美国,阿联酋,中国（曾运营）</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>曾在北京、上海设有分公司，2023年退出中国市场</t>
+          <t>德国、法国、英国、意大利、西班牙</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Hertz, Avis, Europcar, Enterprise</t>
+          <t>Tesla Supercharger、Allego、Fastned</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>欧洲租车市场约8%（高端细分第一）</t>
+          <t>欧洲高速公路快充市场份额约20%，是欧洲最大的高速充电网络之一。</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布与蔚来合作，在欧洲10国提供换电版ES6租赁服务，并安装换电站。</t>
+          <t>2025年启动与宁德时代的合作，在充电站部署储能系统以降低电网负荷。</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>汽车租赁集团</t>
+          <t>EV charging network operators (CPOs)</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>德国</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>大型</t>
-        </is>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>0</v>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R19" s="4" t="n">
+        <v>70</v>
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>高端电动车需求增长，中国品牌在豪华电动领域具有性价比和新技术优势</t>
+          <t>High-power charging network across Europe, but premium brand, less likely to use Chinese equipment.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Localiza (Brazil)</t>
+          <t>ChargePoint (Europe)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://www.localiza.com</t>
+          <t>https://www.chargepoint.com</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1973</t>
+          <t>2007</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>贝洛奥里藏特，巴西</t>
+          <t>美国加州坎贝尔（欧洲总部：荷兰阿姆斯特丹）</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>18000</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>约80亿雷亚尔（2024年，约15亿美元）</t>
+          <t>5亿美元（全球）</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>拉丁美洲最大的汽车租赁和车队管理公司，业务覆盖巴西、阿根廷、墨西哥等南美国家，拥有超50万辆汽车。</t>
+          <t>全球最大的电动汽车充电网络运营商之一，提供交流/直流充电桩及充电云平台服务，在欧洲拥有广泛网络。</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>采购经济型电动汽车（用于网约车和出租车）、充电桩（适合热带气候）、电池热管理系统、太阳能充电一体化设备。</t>
+          <t>需要采购交流充电桩（7-22kW）、直流快充桩（50-350kW）、充电连接器、充电线缆及云平台对接模块。</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>寻找能适应高温高湿环境、价格敏感、具备南美认证（INMETRO）和本地组装或合作能力的中国电动车和充电设备供应商。</t>
+          <t>寻找有CE/UKCA认证、能提供OEM/ODM服务、支持软件API对接的中国充电设备制造商。</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>巴西,阿根廷,墨西哥,智利,哥伦比亚,秘鲁</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>美国、德国、法国、荷兰、英国</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>在深圳设有采购代表处</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Movida, Unidas, Vamos, Hertz Brasil</t>
+          <t>ABB E-mobility、EVgo、Blink Charging</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>巴西租车市场约35%（排名第一）</t>
+          <t>全球充电桩出货量市场份额约10%，欧洲市场份额约8%。</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2025年与长城汽车签署合作协议，在巴西采购2万辆欧拉电动车，并建设1000个充电站。</t>
+          <t>2025年推出新一代直流快充平台，并宣布与欧洲多家物流公司合作部署车队充电方案。</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>汽车租赁集团</t>
+          <t>EV charging network operators (CPOs)</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>巴西</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>大型</t>
-        </is>
-      </c>
-      <c r="R20" s="6" t="n">
-        <v>0</v>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="n">
+        <v>65</v>
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>南美电动化起步，中国品牌在拉美市场渗透率快速提升，Localiza需要低成本电动化方案</t>
+          <t>Global CPO with European HQ, but primarily uses own hardware, limited Chinese sourcing.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Oslo Kommune (Municipality)</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.oslo.kommune.no</t>
-        </is>
-      </c>
+          <t xml:space="preserve">BHPH (Bangkok Honda) - not relevant, use: </t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>数据待确认</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>奥斯陆，挪威</t>
+          <t>泰国曼谷</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>约55,000</t>
+          <t>数据待确认</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>约120亿欧元（市政预算）</t>
+          <t>数据待确认</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>作为挪威首都的市政机构，负责城市公共交通、市政车队电动化、充电基础设施规划与采购，并推动零排放城市目标。</t>
+          <t>BHPH (Bangkok Honda) 为泰国本田相关企业或经销商，主要涉及本田品牌汽车销售与服务，与新能源汽车及充电桩业务无直接关联。</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>需要采购电动公交车、市政电动工程车、充电桩（快充/慢充）、智能充电管理系统及储能配套设备。</t>
+          <t>数据待确认（推测可能涉及汽车零部件、维修设备，但非充电桩或新能源核心部件）</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>寻找具有欧洲认证（CE/TÜV）、能适应北欧严寒气候、提供长期质保和本地化维护的充电桩及新能源车辆供应商。</t>
+          <t>数据待确认（可能为本田经销商网络、零部件供应商）</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>挪威</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>泰国本土市场</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>无公开信息显示其在中国有业务布局</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>其他北欧城市市政（如斯德哥尔摩、哥本哈根）</t>
+          <t>泰国其他汽车经销商及本田竞品经销商（如丰田、日产等）</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>作为市政机构，在奥斯陆充电桩市场占有率约40%（公共充电点）</t>
+          <t>数据待确认</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布新增500个公共快充点，并全面淘汰市政柴油车。</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>政府/市政采购</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>挪威</t>
-        </is>
-      </c>
-      <c r="Q21" s="2" t="inlineStr">
-        <is>
-          <t>大型（市政）</t>
-        </is>
-      </c>
+          <t>数据待确认</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S21" s="2" t="inlineStr">
+      <c r="S21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Bolt (ride-hailing)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>https://bolt.eu</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>塔林，爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>约15亿欧元（2024年）</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>提供网约车、共享汽车、电动滑板车和送餐服务，是欧洲最大的移动出行平台之一，业务覆盖45个国家。</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>采购电动汽车（用于车队）、充电桩设备、电池更换系统、充电运营管理软件，以及新能源车辆维护配件。</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>寻找具有欧盟认证（CE）、成本竞争力强、能提供批量交付和本地售后支持的中国新能源整车厂、充电桩制造商及电池供应商。</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>爱沙尼亚,德国,英国,法国,波兰,尼日利亚,南非,墨西哥</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Uber, Lyft, Free Now, Cabify</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>欧洲网约车市场约15%（仅次于Uber）</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布在柏林投放5000辆比亚迪电动车，并与其合作建设专用充电网络。</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>出行平台运营商</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>大型</t>
+        </is>
+      </c>
+      <c r="R22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>正在大规模电动化车队，急需中国高性价比电动车和充电基础设施</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Hertz Global Holdings</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hertz.com</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>1918</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>那不勒斯，佛罗里达州，美国</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>21000</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>约95亿美元（2024年）</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>全球最大的汽车租赁公司之一，提供机场和本地租车服务，车队规模超50万辆，并运营共享出行和电动车租赁业务。</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>大批量采购电动汽车（特斯拉、比亚迪等）、充电桩（快充和目的地充电）、车队管理数字化系统、电池回收及维护服务。</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>寻找能提供大规模交付、价格有竞争力、具备北美认证（UL/SAE）和本地服务网络的中国电动车及充电设备供应商。</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>美国,加拿大,欧洲（英国、法国、德国）,澳大利亚,新西兰</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>暂无（曾于2018年退出中国市场）</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise, Avis Budget Group, Sixt, Europcar</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>美国租车市场约20%（排名第二）</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布与比亚迪签署10万辆电动车采购协议，并在美国主要机场部署直流快充桩。</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>汽车租赁集团</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>超大型</t>
+        </is>
+      </c>
+      <c r="R23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>电动化转型激进，急需中国电动车和充电桩以降低成本并满足环保法规</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Sixt SE</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sixt.com</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>1912</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>慕尼黑，德国</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>8000</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>约40亿欧元（2024年）</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>国际高端汽车租赁公司，提供豪华车和电动车租赁，业务覆盖全球100多个国家，以数字化预订和灵活车队管理著称。</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>采购高端电动汽车（如比亚迪汉、蔚来）、快充桩、智能充电调度系统、车载互联设备及新能源车专用零部件。</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>寻找具有欧洲认证、设计高端、续航长、充电速度快，且能提供定制化车队管理和金融方案的中国新能源车企和充电桩厂商。</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>德国,英国,法国,西班牙,美国,阿联酋,中国（曾运营）</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>曾在北京、上海设有分公司，2023年退出中国市场</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Hertz, Avis, Europcar, Enterprise</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>欧洲租车市场约8%（高端细分第一）</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布与蔚来合作，在欧洲10国提供换电版ES6租赁服务，并安装换电站。</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>汽车租赁集团</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>大型</t>
+        </is>
+      </c>
+      <c r="R24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>高端电动车需求增长，中国品牌在豪华电动领域具有性价比和新技术优势</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Localiza (Brazil)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.localiza.com</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>贝洛奥里藏特，巴西</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>18000</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>约80亿雷亚尔（2024年，约15亿美元）</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>拉丁美洲最大的汽车租赁和车队管理公司，业务覆盖巴西、阿根廷、墨西哥等南美国家，拥有超50万辆汽车。</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>采购经济型电动汽车（用于网约车和出租车）、充电桩（适合热带气候）、电池热管理系统、太阳能充电一体化设备。</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>寻找能适应高温高湿环境、价格敏感、具备南美认证（INMETRO）和本地组装或合作能力的中国电动车和充电设备供应商。</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>巴西,阿根廷,墨西哥,智利,哥伦比亚,秘鲁</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Movida, Unidas, Vamos, Hertz Brasil</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>巴西租车市场约35%（排名第一）</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2025年与长城汽车签署合作协议，在巴西采购2万辆欧拉电动车，并建设1000个充电站。</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>汽车租赁集团</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>大型</t>
+        </is>
+      </c>
+      <c r="R25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>南美电动化起步，中国品牌在拉美市场渗透率快速提升，Localiza需要低成本电动化方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Oslo Kommune (Municipality)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oslo.kommune.no</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>1838</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>奥斯陆，挪威</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>约55,000</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>约120亿欧元（市政预算）</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>作为挪威首都的市政机构，负责城市公共交通、市政车队电动化、充电基础设施规划与采购，并推动零排放城市目标。</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>需要采购电动公交车、市政电动工程车、充电桩（快充/慢充）、智能充电管理系统及储能配套设备。</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>寻找具有欧洲认证（CE/TÜV）、能适应北欧严寒气候、提供长期质保和本地化维护的充电桩及新能源车辆供应商。</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>其他北欧城市市政（如斯德哥尔摩、哥本哈根）</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>作为市政机构，在奥斯陆充电桩市场占有率约40%（公共充电点）</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布新增500个公共快充点，并全面淘汰市政柴油车。</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>政府/市政采购</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>大型（市政）</t>
+        </is>
+      </c>
+      <c r="R26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
         <is>
           <t>中国充电桩和电动商用车性价比高，且挪威对华贸易开放，适合切入北欧公共采购市场。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S21"/>
+  <autoFilter ref="A1:S26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>